<commit_message>
Pubs premium : 5 miniatures + textes Meta des 5 films dans le kit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRiR3Ga39EKt9eeNc8DXDQ
</commit_message>
<xml_diff>
--- a/LIMO-video/pub-ads/KIT-PUB-LIMO.xlsx
+++ b/LIMO-video/pub-ads/KIT-PUB-LIMO.xlsx
@@ -3236,7 +3236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3323,20 +3323,281 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
+          <t>A – Premium</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>premium-pack/prem-02-trois-erreurs.mp4</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Liste · 3 erreurs (40 s)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Conseiller immo, voici 3 erreurs qui te font perdre des mandats 👇
+1️⃣ Tu rappelles trop tard après l'estimation
+2️⃣ Tes relances sont dans ta tête
+3️⃣ Tes soirées partent dans l'administratif
+Limo corrige les trois. Essai gratuit 14 jours, sans carte bancaire.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Ne perds plus un mandat par oubli</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Le bras droit du conseiller immo</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>S'inscrire</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=prem-trois-erreurs</t>
+        </is>
+      </c>
+      <c r="J5" s="5">
+        <f>LEN(F5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="190" customHeight="1">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>A – Premium</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>premium-pack/prem-03-dimanche-soir.mp4</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>POV · dimanche soir (23 s)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Dimanche, 22 h. Tu ressors tes notes pour savoir qui rappeler… 😩
+Ton collègue, lui, regarde un film. Son secret ? Limo prépare sa semaine : relances, rendez-vous, dossiers.
+Reprends tes dimanches. 14 jours offerts, sans CB.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Reprends tes dimanches</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Essai gratuit 14 jours</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>S'inscrire</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=prem-dimanche-soir</t>
+        </is>
+      </c>
+      <c r="J6" s="5">
+        <f>LEN(F6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="190" customHeight="1">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>A – Premium</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>premium-pack/prem-04-le-calcul.mp4</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Rationnel · le calcul (28 s)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Fais le calcul : 1 h d'administratif par jour, c'est plus de 200 h par an ⏱️
+Limo s'occupe des relances, des comptes rendus, des annonces et du suivi des dossiers. Toi, tu retournes sur le terrain.
+Dès 49 €/mois · essai 14 jours sans carte bancaire.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Récupère tes heures d'admin</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Dès 49 €/mois · sans engagement</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>S'inscrire</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=prem-le-calcul</t>
+        </is>
+      </c>
+      <c r="J7" s="5">
+        <f>LEN(F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="190" customHeight="1">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>A – Premium (vague 2)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>premium-pack/prem-01-regarde-ca.mp4</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Démo · regarde ça (30 s)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Conseiller immo, regarde ça 👀
+Tu demandes « rappelle-moi le bien de M. et Mme T. »… et Limo te sort tout : documents, propriétaires, estimation, diagnostics.
+Pendant ce temps, il relance tes acquéreurs, ton diagnostiqueur et complète le dossier notaire.
+Teste-le 14 jours, sans carte bancaire.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Ton assistant connaît tes biens</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Essai gratuit 14 jours</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>S'inscrire</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=prem-regarde-ca</t>
+        </is>
+      </c>
+      <c r="J8" s="5">
+        <f>LEN(F8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="190" customHeight="1">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>A – Premium (vague 2)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>premium-pack/prem-05-une-journee.mp4</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Démo · une journée (34 s)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>8 h : tes priorités sont prêtes.
+10 h : tu dictes ton compte rendu dans la voiture, la fiche est créée.
+14 h : nouveau mandat ? L'annonce est rédigée en 2 minutes.
+18 h : diagnostiqueur relancé, notaire servi.
+Et toi ? Tu as passé ta journée avec tes clients. 🏡
+Limo, le bras droit du conseiller immo. Essai gratuit 14 jours.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Une journée avec Limo</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Le bras droit du conseiller immo</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>S'inscrire</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=prem-une-journee</t>
+        </is>
+      </c>
+      <c r="J9" s="5">
+        <f>LEN(F9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="190" customHeight="1">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
           <t>A – Acquisition</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>voix/voix-03-surcharge.mp4</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>Surcharge (10 s)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Conseiller immo, surchargé ?
 Appels manqués, relances oubliées, dossiers incomplets… LIMO s'en occupe pour toi.
@@ -3346,51 +3607,51 @@
 Essai gratuit 14 jours, sans carte bancaire.</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>LIMO, le bras droit du conseiller</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Dès 49 €/mois · sans engagement</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>S'inscrire</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=surcharge</t>
         </is>
       </c>
-      <c r="J5" s="5">
-        <f>LEN(F5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="190" customHeight="1">
-      <c r="A6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="J10" s="5">
+        <f>LEN(F10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="190" customHeight="1">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>A – Acquisition</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>voix/voix-01-julien.mp4</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Storytelling (59 s)</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Julien a fait une super estimation. Puis il a oublié de rappeler.
 Quelques jours plus tard, un autre panneau était sur la maison.
@@ -3399,51 +3660,51 @@
 👉 Réserve ta démo de 15 min.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Ne perds plus un mandat par oubli</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Démo gratuite de 15 min</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Réserver</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=julien</t>
         </is>
       </c>
-      <c r="J6" s="5">
-        <f>LEN(F6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="190" customHeight="1">
-      <c r="A7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="J11" s="5">
+        <f>LEN(F11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="190" customHeight="1">
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>A – Acquisition</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>voix/voix-02-regarde-ca.mp4</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Démo produit (30 s)</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Conseiller immo, regarde ça 👀
 Tu demandes « rappelle-moi le bien de M. et Mme T. » → LIMO te sort la fiche complète : documents, diagnostics, propriétaires, estimation.
@@ -3451,51 +3712,51 @@
 Teste-le 14 jours, sans CB.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Toute ton activité, au même endroit</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Essai gratuit 14 jours</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>S'inscrire</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=regarde-ca</t>
         </is>
       </c>
-      <c r="J7" s="5">
-        <f>LEN(F7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="190" customHeight="1">
-      <c r="A8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="J12" s="5">
+        <f>LEN(F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="190" customHeight="1">
+      <c r="A13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>A – Acquisition</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>pubs-30s/LIMO-pub30-01-mandats-perdus-9x16.mp4</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Perte de mandats (30 s)</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Combien de mandats as-tu perdus cette année… juste par manque de suivi ?
 LIMO relance tes vendeurs au bon moment, prépare tes estimations et garde tous tes dossiers à jour.
@@ -3503,51 +3764,51 @@
 Essai gratuit 14 jours, sans carte bancaire.</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Arrête de perdre des mandats</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Dès 49 €/mois</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>S'inscrire</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=mandats-perdus</t>
         </is>
       </c>
-      <c r="J8" s="5">
-        <f>LEN(F8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="190" customHeight="1">
-      <c r="A9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="J13" s="5">
+        <f>LEN(F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="190" customHeight="1">
+      <c r="A14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>A – Acquisition</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>lifestyle/LIMO-life-02-pov-collegue-9x16.mp4</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>POV / humour</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>POV : ton collègue a l'air moins débordé que toi… et il rentre plus tôt 😅
 Son secret ? LIMO, le bras droit du conseiller immo.
@@ -3555,51 +3816,51 @@
 14 jours pour tester, sans CB.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Son secret ? LIMO.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Essai gratuit 14 jours</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>En savoir plus</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=acquisition&amp;utm_content=pov-collegue</t>
         </is>
       </c>
-      <c r="J9" s="5">
-        <f>LEN(F9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="190" customHeight="1">
-      <c r="A10" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="J14" s="5">
+        <f>LEN(F14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="190" customHeight="1">
+      <c r="A15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>B – Relance</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>signatures/sign-01-derriere-chaque-signature.mp4</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Émotion (32 s)</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Le jour de la signature, on oublie tout le reste.
 Les appels du soir, les relances, les compromis, les diagnostics, les échanges avec le notaire…
@@ -3607,108 +3868,108 @@
 👉 Réserve ta démo de 15 min.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Du mandat à la signature, sans oubli</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Démo gratuite de 15 min</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>Réserver</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=relance&amp;utm_content=signatures</t>
         </is>
       </c>
-      <c r="J10" s="5">
-        <f>LEN(F10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="190" customHeight="1">
-      <c r="A11" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="J15" s="5">
+        <f>LEN(F15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="190" customHeight="1">
+      <c r="A16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>B – Relance</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>cine/LIMO-cine-03-le-calcul-9x16.mp4</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Rationnel (temps/argent)</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Fais le calcul : combien d'heures par semaine passes-tu sur l'administratif ?
 LIMO te les rend : relances, dossiers, annonces et estimations automatisés.
 Tu as déjà vu LIMO passer. Il ne te reste qu'à l'essayer : 14 jours, sans carte bancaire.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Récupère tes heures d'admin</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Dès 49 €/mois · sans engagement</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>S'inscrire</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>https://app.leadengineai.fr/?utm_source=meta&amp;utm_medium=paid_social&amp;utm_campaign=relance&amp;utm_content=le-calcul</t>
         </is>
       </c>
-      <c r="J11" s="5">
-        <f>LEN(F11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="J16" s="5">
+        <f>LEN(F16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Réglages campagne A</t>
         </is>
       </c>
-      <c r="E13" s="35" t="inlineStr">
+      <c r="E18" s="35" t="inlineStr">
         <is>
           <t>Objectif Ventes · Conversion : CompleteRegistration · France · 25-60 ans · ciblage large (Advantage+) · placements Advantage+ · 20 €/jour · ne rien modifier 5-7 jours</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="6" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Réglages campagne B</t>
         </is>
       </c>
-      <c r="E14" s="35" t="inlineStr">
+      <c r="E19" s="35" t="inlineStr">
         <is>
           <t>Objectif Prospects · Conversion : Lead · Audiences : vidéo vue à 50 % + interactions Page/Insta + visiteurs site 30 j · EXCLURE les inscrits · 5-8 €/jour</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J5:J11">
+  <conditionalFormatting sqref="J5:J16">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="2">
       <formula>40</formula>
     </cfRule>

</xml_diff>